<commit_message>
chore: Update GitHub Actions to publish detailed Selenium E2E artifacts
</commit_message>
<xml_diff>
--- a/test-reports/Selenium_E2E_300_TestCases_Analysis_Report.xlsx
+++ b/test-reports/Selenium_E2E_300_TestCases_Analysis_Report.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45.83203125" customWidth="1" min="1" max="1"/>
@@ -464,7 +464,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -565,7 +564,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -938,6 +936,69 @@
       <c r="F26" t="inlineStr">
         <is>
           <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AUTOMATED E2E SELENIUM TEST RUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-08-17 09:44:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Total Detailed Scenarios Executed</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Pass Rate</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Detailed Log</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Saved in selenium-tests/Selenium_E2E_Detailed_Test_Report.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>